<commit_message>
data(employees): collapse to canonical 5 professions + V/X availability
The user reorganized av.xlsx (now uses V/X cells throughout) and asked
us to fold the detailed military specialties into our 5-profession
canonical list: רכב / טנק / מנהל / מחסנאי / נשק.

Mapping applied:
  קצינים   → מנהל  (also permissions=manager — these are officers)
  מכונאות / בק״ש / חשמל / צריח / חילוץ / א.נ.ם → טנק
  רכב      → רכב
  נשק      → נשק

Headcount after collapse:
  טנק:   16
  רכב:    5
  נשק:    3
  מנהל:   2
  מחסנאי: 0  (no source role; will be assigned manually)

Stable employee numbering: NAME_NUMBER map keyed by name (in the
original group order from the first av.xlsx). Re-runs of the script
on a re-ordered av.xlsx keep the same numbers per person.

Availability classifier simplified to V/X (case-insensitive). Empty
cells default to V. Result: 1326 V + 572 X = 1898 (26×73).

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/worker_templates/employee_availability.xlsx
+++ b/worker_templates/employee_availability.xlsx
@@ -908,7 +908,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -978,7 +978,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -1033,22 +1033,22 @@
       </c>
       <c r="AC2" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
@@ -1103,22 +1103,22 @@
       </c>
       <c r="AQ2" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AR2" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AS2" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AT2" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AU2" t="inlineStr">
@@ -1173,22 +1173,22 @@
       </c>
       <c r="BE2" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BF2" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BG2" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BH2" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BI2" t="inlineStr">
@@ -1303,22 +1303,22 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -1328,7 +1328,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>V</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -1373,22 +1373,22 @@
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="Z3" t="inlineStr">
@@ -1443,22 +1443,22 @@
       </c>
       <c r="AJ3" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AK3" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AL3" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AM3" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AN3" t="inlineStr">
@@ -1513,22 +1513,22 @@
       </c>
       <c r="AX3" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AY3" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AZ3" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BA3" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BB3" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="BL3" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BM3" t="inlineStr">
@@ -1653,12 +1653,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -1713,22 +1713,22 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -1783,22 +1783,22 @@
       </c>
       <c r="AC4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AD4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AE4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AF4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AG4" t="inlineStr">
@@ -1828,7 +1828,7 @@
       </c>
       <c r="AL4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>V</t>
         </is>
       </c>
       <c r="AM4" t="inlineStr">
@@ -1853,22 +1853,22 @@
       </c>
       <c r="AQ4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AR4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AS4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AT4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AU4" t="inlineStr">
@@ -1923,22 +1923,22 @@
       </c>
       <c r="BE4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BF4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BG4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BH4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BI4" t="inlineStr">
@@ -2028,12 +2028,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -2088,22 +2088,22 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -2158,22 +2158,22 @@
       </c>
       <c r="AC5" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AD5" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AE5" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AG5" t="inlineStr">
@@ -2228,22 +2228,22 @@
       </c>
       <c r="AQ5" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AR5" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AS5" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AT5" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AU5" t="inlineStr">
@@ -2298,22 +2298,22 @@
       </c>
       <c r="BE5" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BF5" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BG5" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BH5" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BI5" t="inlineStr">
@@ -2403,7 +2403,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>V</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -2443,7 +2443,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -2453,7 +2453,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>V</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -2498,22 +2498,22 @@
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="Y6" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="Z6" t="inlineStr">
@@ -2568,22 +2568,22 @@
       </c>
       <c r="AJ6" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AK6" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AL6" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AM6" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AN6" t="inlineStr">
@@ -2608,7 +2608,7 @@
       </c>
       <c r="AR6" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>V</t>
         </is>
       </c>
       <c r="AS6" t="inlineStr">
@@ -2638,22 +2638,22 @@
       </c>
       <c r="AX6" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AY6" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AZ6" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BA6" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BB6" t="inlineStr">
@@ -2708,7 +2708,7 @@
       </c>
       <c r="BL6" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BM6" t="inlineStr">
@@ -2778,12 +2778,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -2838,22 +2838,22 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -2903,27 +2903,27 @@
       </c>
       <c r="AB7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AC7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AD7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AE7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AF7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AG7" t="inlineStr">
@@ -2978,22 +2978,22 @@
       </c>
       <c r="AQ7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AR7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AS7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AT7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AU7" t="inlineStr">
@@ -3048,22 +3048,22 @@
       </c>
       <c r="BE7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BF7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BG7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BH7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BI7" t="inlineStr">
@@ -3178,22 +3178,22 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -3248,22 +3248,22 @@
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="W8" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="Y8" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="Z8" t="inlineStr">
@@ -3318,22 +3318,22 @@
       </c>
       <c r="AJ8" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AK8" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AL8" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AM8" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AN8" t="inlineStr">
@@ -3388,22 +3388,22 @@
       </c>
       <c r="AX8" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AY8" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AZ8" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BA8" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BB8" t="inlineStr">
@@ -3458,7 +3458,7 @@
       </c>
       <c r="BL8" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BM8" t="inlineStr">
@@ -3548,27 +3548,27 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -3623,22 +3623,22 @@
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="W9" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="Y9" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="Z9" t="inlineStr">
@@ -3693,22 +3693,22 @@
       </c>
       <c r="AJ9" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AK9" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AL9" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AM9" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AN9" t="inlineStr">
@@ -3763,22 +3763,22 @@
       </c>
       <c r="AX9" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AY9" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AZ9" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BA9" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BB9" t="inlineStr">
@@ -3833,7 +3833,7 @@
       </c>
       <c r="BL9" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BM9" t="inlineStr">
@@ -3878,7 +3878,7 @@
       </c>
       <c r="BU9" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>V</t>
         </is>
       </c>
       <c r="BV9" t="inlineStr">
@@ -3903,12 +3903,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -3963,22 +3963,22 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -4033,22 +4033,22 @@
       </c>
       <c r="AC10" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AD10" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AE10" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AF10" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AG10" t="inlineStr">
@@ -4103,22 +4103,22 @@
       </c>
       <c r="AQ10" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AR10" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AS10" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AT10" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AU10" t="inlineStr">
@@ -4173,22 +4173,22 @@
       </c>
       <c r="BE10" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BF10" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BG10" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BH10" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BI10" t="inlineStr">
@@ -4303,22 +4303,22 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -4373,22 +4373,22 @@
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="W11" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="Y11" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="Z11" t="inlineStr">
@@ -4443,22 +4443,22 @@
       </c>
       <c r="AJ11" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AK11" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AL11" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AM11" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AN11" t="inlineStr">
@@ -4513,22 +4513,22 @@
       </c>
       <c r="AX11" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AY11" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AZ11" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BA11" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BB11" t="inlineStr">
@@ -4583,7 +4583,7 @@
       </c>
       <c r="BL11" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BM11" t="inlineStr">
@@ -4673,27 +4673,27 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -4748,22 +4748,22 @@
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="W12" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="Y12" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="Z12" t="inlineStr">
@@ -4818,22 +4818,22 @@
       </c>
       <c r="AJ12" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AK12" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AL12" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AM12" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AN12" t="inlineStr">
@@ -4888,22 +4888,22 @@
       </c>
       <c r="AX12" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AY12" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AZ12" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BA12" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BB12" t="inlineStr">
@@ -4958,7 +4958,7 @@
       </c>
       <c r="BL12" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BM12" t="inlineStr">
@@ -5003,7 +5003,7 @@
       </c>
       <c r="BU12" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>V</t>
         </is>
       </c>
       <c r="BV12" t="inlineStr">
@@ -5028,12 +5028,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -5088,12 +5088,12 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
@@ -5158,22 +5158,22 @@
       </c>
       <c r="AC13" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AD13" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AE13" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AF13" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AG13" t="inlineStr">
@@ -5228,22 +5228,22 @@
       </c>
       <c r="AQ13" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AR13" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AS13" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AT13" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AU13" t="inlineStr">
@@ -5298,22 +5298,22 @@
       </c>
       <c r="BE13" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BF13" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BG13" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BH13" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BI13" t="inlineStr">
@@ -5423,27 +5423,27 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -5498,22 +5498,22 @@
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="W14" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="Y14" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="Z14" t="inlineStr">
@@ -5568,22 +5568,22 @@
       </c>
       <c r="AJ14" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AK14" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AL14" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AM14" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AN14" t="inlineStr">
@@ -5638,22 +5638,22 @@
       </c>
       <c r="AX14" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AY14" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AZ14" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BA14" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BB14" t="inlineStr">
@@ -5708,7 +5708,7 @@
       </c>
       <c r="BL14" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BM14" t="inlineStr">
@@ -5753,7 +5753,7 @@
       </c>
       <c r="BU14" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>V</t>
         </is>
       </c>
       <c r="BV14" t="inlineStr">
@@ -5798,27 +5798,27 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -5873,22 +5873,22 @@
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="Z15" t="inlineStr">
@@ -5943,22 +5943,22 @@
       </c>
       <c r="AJ15" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AK15" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AL15" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AM15" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AN15" t="inlineStr">
@@ -6013,22 +6013,22 @@
       </c>
       <c r="AX15" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AY15" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AZ15" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BA15" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BB15" t="inlineStr">
@@ -6083,7 +6083,7 @@
       </c>
       <c r="BL15" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BM15" t="inlineStr">
@@ -6128,7 +6128,7 @@
       </c>
       <c r="BU15" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>V</t>
         </is>
       </c>
       <c r="BV15" t="inlineStr">
@@ -6153,12 +6153,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -6213,22 +6213,22 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -6283,22 +6283,22 @@
       </c>
       <c r="AC16" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AD16" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AE16" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AF16" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AG16" t="inlineStr">
@@ -6353,22 +6353,22 @@
       </c>
       <c r="AQ16" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AR16" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AS16" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AT16" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AU16" t="inlineStr">
@@ -6423,22 +6423,22 @@
       </c>
       <c r="BE16" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BF16" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BG16" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BH16" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BI16" t="inlineStr">
@@ -6553,22 +6553,22 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -6623,22 +6623,22 @@
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="Z17" t="inlineStr">
@@ -6693,22 +6693,22 @@
       </c>
       <c r="AJ17" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AK17" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AL17" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AM17" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AN17" t="inlineStr">
@@ -6763,22 +6763,22 @@
       </c>
       <c r="AX17" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AY17" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AZ17" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BA17" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BB17" t="inlineStr">
@@ -6833,7 +6833,7 @@
       </c>
       <c r="BL17" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BM17" t="inlineStr">
@@ -6903,12 +6903,12 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -6963,22 +6963,22 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -7033,22 +7033,22 @@
       </c>
       <c r="AC18" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AD18" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AE18" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AF18" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AG18" t="inlineStr">
@@ -7103,27 +7103,27 @@
       </c>
       <c r="AQ18" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AR18" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AS18" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AT18" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AU18" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>V</t>
         </is>
       </c>
       <c r="AV18" t="inlineStr">
@@ -7173,22 +7173,22 @@
       </c>
       <c r="BE18" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BF18" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BG18" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BH18" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BI18" t="inlineStr">
@@ -7278,12 +7278,12 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -7338,22 +7338,22 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -7408,22 +7408,22 @@
       </c>
       <c r="AC19" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AD19" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AE19" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AF19" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AG19" t="inlineStr">
@@ -7473,7 +7473,7 @@
       </c>
       <c r="AP19" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AQ19" t="inlineStr">
@@ -7483,17 +7483,17 @@
       </c>
       <c r="AR19" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AS19" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AT19" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AU19" t="inlineStr">
@@ -7548,22 +7548,22 @@
       </c>
       <c r="BE19" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BF19" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BG19" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BH19" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BI19" t="inlineStr">
@@ -7688,12 +7688,12 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
@@ -7748,22 +7748,22 @@
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="Z20" t="inlineStr">
@@ -7818,22 +7818,22 @@
       </c>
       <c r="AJ20" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AK20" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AL20" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AM20" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AN20" t="inlineStr">
@@ -7888,22 +7888,22 @@
       </c>
       <c r="AX20" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AY20" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AZ20" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BA20" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BB20" t="inlineStr">
@@ -7948,12 +7948,12 @@
       </c>
       <c r="BJ20" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>V</t>
         </is>
       </c>
       <c r="BK20" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BL20" t="inlineStr">
@@ -8053,22 +8053,22 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -8123,22 +8123,22 @@
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="Z21" t="inlineStr">
@@ -8193,22 +8193,22 @@
       </c>
       <c r="AJ21" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AK21" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AL21" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AM21" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AN21" t="inlineStr">
@@ -8263,22 +8263,22 @@
       </c>
       <c r="AX21" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AY21" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AZ21" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BA21" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BB21" t="inlineStr">
@@ -8333,7 +8333,7 @@
       </c>
       <c r="BL21" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BM21" t="inlineStr">
@@ -8403,12 +8403,12 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -8463,22 +8463,22 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -8533,22 +8533,22 @@
       </c>
       <c r="AC22" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AD22" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AE22" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AF22" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AG22" t="inlineStr">
@@ -8603,22 +8603,22 @@
       </c>
       <c r="AQ22" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AR22" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AS22" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AT22" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AU22" t="inlineStr">
@@ -8653,7 +8653,7 @@
       </c>
       <c r="BA22" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>V</t>
         </is>
       </c>
       <c r="BB22" t="inlineStr">
@@ -8673,22 +8673,22 @@
       </c>
       <c r="BE22" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BF22" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BG22" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BH22" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BI22" t="inlineStr">
@@ -8803,22 +8803,22 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
@@ -8873,22 +8873,22 @@
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="Z23" t="inlineStr">
@@ -8943,22 +8943,22 @@
       </c>
       <c r="AJ23" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AK23" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AL23" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AM23" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AN23" t="inlineStr">
@@ -9013,22 +9013,22 @@
       </c>
       <c r="AX23" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AY23" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AZ23" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BA23" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BB23" t="inlineStr">
@@ -9083,7 +9083,7 @@
       </c>
       <c r="BL23" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BM23" t="inlineStr">
@@ -9153,12 +9153,12 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -9218,12 +9218,12 @@
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
@@ -9283,22 +9283,22 @@
       </c>
       <c r="AC24" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AD24" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AE24" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AF24" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AG24" t="inlineStr">
@@ -9353,22 +9353,22 @@
       </c>
       <c r="AQ24" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AR24" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AS24" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AT24" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AU24" t="inlineStr">
@@ -9423,22 +9423,22 @@
       </c>
       <c r="BE24" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BF24" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BG24" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BH24" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BI24" t="inlineStr">
@@ -9533,7 +9533,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -9603,7 +9603,7 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
@@ -9658,22 +9658,22 @@
       </c>
       <c r="AC25" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AD25" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AE25" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AF25" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AG25" t="inlineStr">
@@ -9728,22 +9728,22 @@
       </c>
       <c r="AQ25" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AR25" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AS25" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AT25" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AU25" t="inlineStr">
@@ -9798,22 +9798,22 @@
       </c>
       <c r="BE25" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BF25" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BG25" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BH25" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BI25" t="inlineStr">
@@ -9928,22 +9928,22 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
@@ -9998,22 +9998,22 @@
       </c>
       <c r="V26" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="W26" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="X26" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="Y26" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="Z26" t="inlineStr">
@@ -10068,22 +10068,22 @@
       </c>
       <c r="AJ26" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AK26" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AL26" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AM26" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AN26" t="inlineStr">
@@ -10138,22 +10138,22 @@
       </c>
       <c r="AX26" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AY26" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AZ26" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BA26" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BB26" t="inlineStr">
@@ -10208,7 +10208,7 @@
       </c>
       <c r="BL26" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BM26" t="inlineStr">
@@ -10278,12 +10278,12 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -10313,7 +10313,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>V</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -10338,22 +10338,22 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
@@ -10408,22 +10408,22 @@
       </c>
       <c r="AC27" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AD27" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AE27" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AF27" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AG27" t="inlineStr">
@@ -10478,22 +10478,22 @@
       </c>
       <c r="AQ27" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AR27" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AS27" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AT27" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="AU27" t="inlineStr">
@@ -10548,22 +10548,22 @@
       </c>
       <c r="BE27" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BF27" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BG27" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BH27" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="BI27" t="inlineStr">
@@ -10653,7 +10653,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -10669,7 +10669,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>טבלת זמינות — חולצה מתוך av.xlsx.</t>
+          <t>טבלת זמינות — חולצה מתוך av.xlsx (ערכי V/X).</t>
         </is>
       </c>
     </row>
@@ -10679,69 +10679,21 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>עמודות:</t>
+          <t xml:space="preserve">  • V = זמין באותו יום.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • מספר עובד / שם עובד — מתאים לערכים ב-employees.xlsx.</t>
+          <t xml:space="preserve">  • X = לא זמין.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • כל יום בטווח 01/05/2026 עד 12/07/2026 = עמודה משלו.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>ערכים בתאים:</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • V = העובד זמין באותו יום.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • X = העובד לא זמין.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>מיפוי המקור (av.xlsx → V/X):</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • 'נוכח' / 'התארגנות' / 'סבב' / שם של עובד אחר / חג / תא ריק → V</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • 'בית' / 'אילוץ' / 'צו סגור' / 'אילוץ - צו סגור' / '-' → X</t>
+          <t xml:space="preserve">  • תא ריק במקור טופל כ-V.</t>
         </is>
       </c>
     </row>

</xml_diff>